<commit_message>
Add web parity test cases (section 51) and refresh the spreadsheet
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TEST_SCENARIOS.xlsx
+++ b/TEST_SCENARIOS.xlsx
@@ -12,7 +12,7 @@
     <sheet name="All tests" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'All tests'!$A$1:$M$608</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'All tests'!$A$1:$M$635</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -619,7 +619,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I51"/>
+  <dimension ref="A1:I52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2543,37 +2543,75 @@
       </c>
     </row>
     <row r="51">
-      <c r="B51" s="7" t="inlineStr">
+      <c r="A51" s="5" t="n">
+        <v>51</v>
+      </c>
+      <c r="B51" s="5" t="inlineStr">
+        <is>
+          <t>WEB APP PARITY  (branch feat/shawn-feedback-web-parity)</t>
+        </is>
+      </c>
+      <c r="C51" s="5">
+        <f>COUNTIF('All tests'!$A:$A,A51)</f>
+        <v/>
+      </c>
+      <c r="D51" s="5">
+        <f>COUNTIFS('All tests'!$A:$A,$A51,'All tests'!$I:$I,"Pass")</f>
+        <v/>
+      </c>
+      <c r="E51" s="5">
+        <f>COUNTIFS('All tests'!$A:$A,$A51,'All tests'!$I:$I,"Fail")</f>
+        <v/>
+      </c>
+      <c r="F51" s="5">
+        <f>COUNTIFS('All tests'!$A:$A,$A51,'All tests'!$I:$I,"Blocked")</f>
+        <v/>
+      </c>
+      <c r="G51" s="5">
+        <f>COUNTIFS('All tests'!$A:$A,$A51,'All tests'!$I:$I,"N/A")</f>
+        <v/>
+      </c>
+      <c r="H51" s="5">
+        <f>C51-SUM(D51:G51)</f>
+        <v/>
+      </c>
+      <c r="I51" s="6">
+        <f>IF(C51=0,0,SUM(D51:G51)/C51)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="B52" s="7" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C51" s="7">
-        <f>SUM(C2:C50)</f>
-        <v/>
-      </c>
-      <c r="D51" s="7">
-        <f>SUM(D2:D50)</f>
-        <v/>
-      </c>
-      <c r="E51" s="7">
-        <f>SUM(E2:E50)</f>
-        <v/>
-      </c>
-      <c r="F51" s="7">
-        <f>SUM(F2:F50)</f>
-        <v/>
-      </c>
-      <c r="G51" s="7">
-        <f>SUM(G2:G50)</f>
-        <v/>
-      </c>
-      <c r="H51" s="7">
-        <f>SUM(H2:H50)</f>
-        <v/>
-      </c>
-      <c r="I51" s="8">
-        <f>IF(C51=0,0,SUM(D51:G51)/C51)</f>
+      <c r="C52" s="7">
+        <f>SUM(C2:C51)</f>
+        <v/>
+      </c>
+      <c r="D52" s="7">
+        <f>SUM(D2:D51)</f>
+        <v/>
+      </c>
+      <c r="E52" s="7">
+        <f>SUM(E2:E51)</f>
+        <v/>
+      </c>
+      <c r="F52" s="7">
+        <f>SUM(F2:F51)</f>
+        <v/>
+      </c>
+      <c r="G52" s="7">
+        <f>SUM(G2:G51)</f>
+        <v/>
+      </c>
+      <c r="H52" s="7">
+        <f>SUM(H2:H51)</f>
+        <v/>
+      </c>
+      <c r="I52" s="8">
+        <f>IF(C52=0,0,SUM(D52:G52)/C52)</f>
         <v/>
       </c>
     </row>
@@ -2588,7 +2626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M608"/>
+  <dimension ref="A1:M635"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -24296,9 +24334,1008 @@
       <c r="L608" s="10" t="inlineStr"/>
       <c r="M608" s="10" t="inlineStr"/>
     </row>
+    <row r="609">
+      <c r="A609" s="10" t="n">
+        <v>51</v>
+      </c>
+      <c r="B609" s="10" t="inlineStr">
+        <is>
+          <t>WEB APP PARITY  (branch feat/shawn-feedback-web-parity)</t>
+        </is>
+      </c>
+      <c r="C609" s="10" t="inlineStr">
+        <is>
+          <t>51.1</t>
+        </is>
+      </c>
+      <c r="D609" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E609" s="10" t="inlineStr">
+        <is>
+          <t>REGISTRATIONS</t>
+        </is>
+      </c>
+      <c r="F609" s="10" t="inlineStr">
+        <is>
+          <t>Tick 2 pending players: ticked cards read "Add 2 to Roster"; a sticky bar shows "2 selected [Clear] [Add 2 to Roster]".</t>
+        </is>
+      </c>
+      <c r="G609" s="10" t="inlineStr"/>
+      <c r="H609" s="10" t="inlineStr"/>
+      <c r="I609" s="10" t="inlineStr"/>
+      <c r="J609" s="10" t="inlineStr"/>
+      <c r="K609" s="10" t="inlineStr"/>
+      <c r="L609" s="10" t="inlineStr"/>
+      <c r="M609" s="10" t="inlineStr"/>
+    </row>
+    <row r="610">
+      <c r="A610" s="10" t="n">
+        <v>51</v>
+      </c>
+      <c r="B610" s="10" t="inlineStr">
+        <is>
+          <t>WEB APP PARITY  (branch feat/shawn-feedback-web-parity)</t>
+        </is>
+      </c>
+      <c r="C610" s="10" t="inlineStr">
+        <is>
+          <t>51.2</t>
+        </is>
+      </c>
+      <c r="D610" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E610" s="10" t="inlineStr">
+        <is>
+          <t>REGISTRATIONS</t>
+        </is>
+      </c>
+      <c r="F610" s="10" t="inlineStr">
+        <is>
+          <t>Click the card's "Add 2 to Roster" -&gt; dialog places BOTH, to a team and to an evaluation; progress reaches 2 of 2.</t>
+        </is>
+      </c>
+      <c r="G610" s="10" t="inlineStr"/>
+      <c r="H610" s="10" t="inlineStr"/>
+      <c r="I610" s="10" t="inlineStr"/>
+      <c r="J610" s="10" t="inlineStr"/>
+      <c r="K610" s="10" t="inlineStr"/>
+      <c r="L610" s="10" t="inlineStr"/>
+      <c r="M610" s="10" t="inlineStr"/>
+    </row>
+    <row r="611">
+      <c r="A611" s="10" t="n">
+        <v>51</v>
+      </c>
+      <c r="B611" s="10" t="inlineStr">
+        <is>
+          <t>WEB APP PARITY  (branch feat/shawn-feedback-web-parity)</t>
+        </is>
+      </c>
+      <c r="C611" s="10" t="inlineStr">
+        <is>
+          <t>51.3</t>
+        </is>
+      </c>
+      <c r="D611" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E611" s="10" t="inlineStr">
+        <is>
+          <t>REGISTRATIONS</t>
+        </is>
+      </c>
+      <c r="F611" s="10" t="inlineStr">
+        <is>
+          <t>Select All selects pending only; Deselect All clears; dismissed players are never counted or placed.</t>
+        </is>
+      </c>
+      <c r="G611" s="10" t="inlineStr"/>
+      <c r="H611" s="10" t="inlineStr"/>
+      <c r="I611" s="10" t="inlineStr"/>
+      <c r="J611" s="10" t="inlineStr"/>
+      <c r="K611" s="10" t="inlineStr"/>
+      <c r="L611" s="10" t="inlineStr"/>
+      <c r="M611" s="10" t="inlineStr"/>
+    </row>
+    <row r="612">
+      <c r="A612" s="10" t="n">
+        <v>51</v>
+      </c>
+      <c r="B612" s="10" t="inlineStr">
+        <is>
+          <t>WEB APP PARITY  (branch feat/shawn-feedback-web-parity)</t>
+        </is>
+      </c>
+      <c r="C612" s="10" t="inlineStr">
+        <is>
+          <t>51.4</t>
+        </is>
+      </c>
+      <c r="D612" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E612" s="10" t="inlineStr">
+        <is>
+          <t>REGISTRATIONS</t>
+        </is>
+      </c>
+      <c r="F612" s="10" t="inlineStr">
+        <is>
+          <t>A single, unticked card still adds just that player.</t>
+        </is>
+      </c>
+      <c r="G612" s="10" t="inlineStr"/>
+      <c r="H612" s="10" t="inlineStr"/>
+      <c r="I612" s="10" t="inlineStr"/>
+      <c r="J612" s="10" t="inlineStr"/>
+      <c r="K612" s="10" t="inlineStr"/>
+      <c r="L612" s="10" t="inlineStr"/>
+      <c r="M612" s="10" t="inlineStr"/>
+    </row>
+    <row r="613">
+      <c r="A613" s="10" t="n">
+        <v>51</v>
+      </c>
+      <c r="B613" s="10" t="inlineStr">
+        <is>
+          <t>WEB APP PARITY  (branch feat/shawn-feedback-web-parity)</t>
+        </is>
+      </c>
+      <c r="C613" s="10" t="inlineStr">
+        <is>
+          <t>51.5</t>
+        </is>
+      </c>
+      <c r="D613" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E613" s="10" t="inlineStr">
+        <is>
+          <t>ROSTERS</t>
+        </is>
+      </c>
+      <c r="F613" s="10" t="inlineStr">
+        <is>
+          <t>Team &gt; Players &gt; Select: checkboxes, Select All = whole team (999 on the test team), Delete Selected (N) with confirmation.</t>
+        </is>
+      </c>
+      <c r="G613" s="10" t="inlineStr"/>
+      <c r="H613" s="10" t="inlineStr"/>
+      <c r="I613" s="10" t="inlineStr"/>
+      <c r="J613" s="10" t="inlineStr"/>
+      <c r="K613" s="10" t="inlineStr"/>
+      <c r="L613" s="10" t="inlineStr"/>
+      <c r="M613" s="10" t="inlineStr"/>
+    </row>
+    <row r="614">
+      <c r="A614" s="10" t="n">
+        <v>51</v>
+      </c>
+      <c r="B614" s="10" t="inlineStr">
+        <is>
+          <t>WEB APP PARITY  (branch feat/shawn-feedback-web-parity)</t>
+        </is>
+      </c>
+      <c r="C614" s="10" t="inlineStr">
+        <is>
+          <t>51.6</t>
+        </is>
+      </c>
+      <c r="D614" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E614" s="10" t="inlineStr">
+        <is>
+          <t>ROSTERS</t>
+        </is>
+      </c>
+      <c r="F614" s="10" t="inlineStr">
+        <is>
+          <t>With a search typed, Select All selects only the matches.</t>
+        </is>
+      </c>
+      <c r="G614" s="10" t="inlineStr"/>
+      <c r="H614" s="10" t="inlineStr"/>
+      <c r="I614" s="10" t="inlineStr"/>
+      <c r="J614" s="10" t="inlineStr"/>
+      <c r="K614" s="10" t="inlineStr"/>
+      <c r="L614" s="10" t="inlineStr"/>
+      <c r="M614" s="10" t="inlineStr"/>
+    </row>
+    <row r="615">
+      <c r="A615" s="10" t="n">
+        <v>51</v>
+      </c>
+      <c r="B615" s="10" t="inlineStr">
+        <is>
+          <t>WEB APP PARITY  (branch feat/shawn-feedback-web-parity)</t>
+        </is>
+      </c>
+      <c r="C615" s="10" t="inlineStr">
+        <is>
+          <t>51.7</t>
+        </is>
+      </c>
+      <c r="D615" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E615" s="10" t="inlineStr">
+        <is>
+          <t>ROSTERS</t>
+        </is>
+      </c>
+      <c r="F615" s="10" t="inlineStr">
+        <is>
+          <t>Leaving the Players tab exits select mode.</t>
+        </is>
+      </c>
+      <c r="G615" s="10" t="inlineStr"/>
+      <c r="H615" s="10" t="inlineStr"/>
+      <c r="I615" s="10" t="inlineStr"/>
+      <c r="J615" s="10" t="inlineStr"/>
+      <c r="K615" s="10" t="inlineStr"/>
+      <c r="L615" s="10" t="inlineStr"/>
+      <c r="M615" s="10" t="inlineStr"/>
+    </row>
+    <row r="616">
+      <c r="A616" s="10" t="n">
+        <v>51</v>
+      </c>
+      <c r="B616" s="10" t="inlineStr">
+        <is>
+          <t>WEB APP PARITY  (branch feat/shawn-feedback-web-parity)</t>
+        </is>
+      </c>
+      <c r="C616" s="10" t="inlineStr">
+        <is>
+          <t>51.8</t>
+        </is>
+      </c>
+      <c r="D616" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E616" s="10" t="inlineStr">
+        <is>
+          <t>ROSTERS</t>
+        </is>
+      </c>
+      <c r="F616" s="10" t="inlineStr">
+        <is>
+          <t>Evaluation roster Select All + Delete Selected: all removed; if some fail the message says "X of Y deleted" and the rest stay selected.</t>
+        </is>
+      </c>
+      <c r="G616" s="10" t="inlineStr"/>
+      <c r="H616" s="10" t="inlineStr"/>
+      <c r="I616" s="10" t="inlineStr"/>
+      <c r="J616" s="10" t="inlineStr"/>
+      <c r="K616" s="10" t="inlineStr"/>
+      <c r="L616" s="10" t="inlineStr"/>
+      <c r="M616" s="10" t="inlineStr"/>
+    </row>
+    <row r="617">
+      <c r="A617" s="10" t="n">
+        <v>51</v>
+      </c>
+      <c r="B617" s="10" t="inlineStr">
+        <is>
+          <t>WEB APP PARITY  (branch feat/shawn-feedback-web-parity)</t>
+        </is>
+      </c>
+      <c r="C617" s="10" t="inlineStr">
+        <is>
+          <t>51.9</t>
+        </is>
+      </c>
+      <c r="D617" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E617" s="10" t="inlineStr">
+        <is>
+          <t>ROSTERS</t>
+        </is>
+      </c>
+      <c r="F617" s="10" t="inlineStr">
+        <is>
+          <t>Airplane mode / offline during delete: readable error.</t>
+        </is>
+      </c>
+      <c r="G617" s="10" t="inlineStr"/>
+      <c r="H617" s="10" t="inlineStr"/>
+      <c r="I617" s="10" t="inlineStr"/>
+      <c r="J617" s="10" t="inlineStr"/>
+      <c r="K617" s="10" t="inlineStr"/>
+      <c r="L617" s="10" t="inlineStr"/>
+      <c r="M617" s="10" t="inlineStr"/>
+    </row>
+    <row r="618">
+      <c r="A618" s="10" t="n">
+        <v>51</v>
+      </c>
+      <c r="B618" s="10" t="inlineStr">
+        <is>
+          <t>WEB APP PARITY  (branch feat/shawn-feedback-web-parity)</t>
+        </is>
+      </c>
+      <c r="C618" s="10" t="inlineStr">
+        <is>
+          <t>51.10</t>
+        </is>
+      </c>
+      <c r="D618" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E618" s="10" t="inlineStr">
+        <is>
+          <t>ROSTERS</t>
+        </is>
+      </c>
+      <c r="F618" s="10" t="inlineStr">
+        <is>
+          <t>Excel with a wrong declared range imports every row (not 1); single Name column; cover sheet first.</t>
+        </is>
+      </c>
+      <c r="G618" s="10" t="inlineStr"/>
+      <c r="H618" s="10" t="inlineStr"/>
+      <c r="I618" s="10" t="inlineStr"/>
+      <c r="J618" s="10" t="inlineStr"/>
+      <c r="K618" s="10" t="inlineStr"/>
+      <c r="L618" s="10" t="inlineStr"/>
+      <c r="M618" s="10" t="inlineStr"/>
+    </row>
+    <row r="619">
+      <c r="A619" s="10" t="n">
+        <v>51</v>
+      </c>
+      <c r="B619" s="10" t="inlineStr">
+        <is>
+          <t>WEB APP PARITY  (branch feat/shawn-feedback-web-parity)</t>
+        </is>
+      </c>
+      <c r="C619" s="10" t="inlineStr">
+        <is>
+          <t>51.11</t>
+        </is>
+      </c>
+      <c r="D619" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E619" s="10" t="inlineStr">
+        <is>
+          <t>ROSTERS</t>
+        </is>
+      </c>
+      <c r="F619" s="10" t="inlineStr">
+        <is>
+          <t>20-row CSV/XLSX into an empty team is much faster than before and the summary matches (20 added, jersey/position saved).</t>
+        </is>
+      </c>
+      <c r="G619" s="10" t="inlineStr"/>
+      <c r="H619" s="10" t="inlineStr"/>
+      <c r="I619" s="10" t="inlineStr"/>
+      <c r="J619" s="10" t="inlineStr"/>
+      <c r="K619" s="10" t="inlineStr"/>
+      <c r="L619" s="10" t="inlineStr"/>
+      <c r="M619" s="10" t="inlineStr"/>
+    </row>
+    <row r="620">
+      <c r="A620" s="10" t="n">
+        <v>51</v>
+      </c>
+      <c r="B620" s="10" t="inlineStr">
+        <is>
+          <t>WEB APP PARITY  (branch feat/shawn-feedback-web-parity)</t>
+        </is>
+      </c>
+      <c r="C620" s="10" t="inlineStr">
+        <is>
+          <t>51.12</t>
+        </is>
+      </c>
+      <c r="D620" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E620" s="10" t="inlineStr">
+        <is>
+          <t>ROSTERS</t>
+        </is>
+      </c>
+      <c r="F620" s="10" t="inlineStr">
+        <is>
+          <t>A bad row is reported while the others import; siblings share one guardian account.</t>
+        </is>
+      </c>
+      <c r="G620" s="10" t="inlineStr"/>
+      <c r="H620" s="10" t="inlineStr"/>
+      <c r="I620" s="10" t="inlineStr"/>
+      <c r="J620" s="10" t="inlineStr"/>
+      <c r="K620" s="10" t="inlineStr"/>
+      <c r="L620" s="10" t="inlineStr"/>
+      <c r="M620" s="10" t="inlineStr"/>
+    </row>
+    <row r="621">
+      <c r="A621" s="10" t="n">
+        <v>51</v>
+      </c>
+      <c r="B621" s="10" t="inlineStr">
+        <is>
+          <t>WEB APP PARITY  (branch feat/shawn-feedback-web-parity)</t>
+        </is>
+      </c>
+      <c r="C621" s="10" t="inlineStr">
+        <is>
+          <t>51.13</t>
+        </is>
+      </c>
+      <c r="D621" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E621" s="10" t="inlineStr">
+        <is>
+          <t>TEAM HUB</t>
+        </is>
+      </c>
+      <c r="F621" s="10" t="inlineStr">
+        <is>
+          <t>Team page header reads "&lt;Team name&gt; Hub"; last tab reads "Options"; ?tab=settings links still open it.</t>
+        </is>
+      </c>
+      <c r="G621" s="10" t="inlineStr"/>
+      <c r="H621" s="10" t="inlineStr"/>
+      <c r="I621" s="10" t="inlineStr"/>
+      <c r="J621" s="10" t="inlineStr"/>
+      <c r="K621" s="10" t="inlineStr"/>
+      <c r="L621" s="10" t="inlineStr"/>
+      <c r="M621" s="10" t="inlineStr"/>
+    </row>
+    <row r="622">
+      <c r="A622" s="10" t="n">
+        <v>51</v>
+      </c>
+      <c r="B622" s="10" t="inlineStr">
+        <is>
+          <t>WEB APP PARITY  (branch feat/shawn-feedback-web-parity)</t>
+        </is>
+      </c>
+      <c r="C622" s="10" t="inlineStr">
+        <is>
+          <t>51.14</t>
+        </is>
+      </c>
+      <c r="D622" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E622" s="10" t="inlineStr">
+        <is>
+          <t>TEAM HUB</t>
+        </is>
+      </c>
+      <c r="F622" s="10" t="inlineStr">
+        <is>
+          <t>Options: Export Team Excel and PDF download; 999 players all in the file; no medical info; special characters preserved.</t>
+        </is>
+      </c>
+      <c r="G622" s="10" t="inlineStr"/>
+      <c r="H622" s="10" t="inlineStr"/>
+      <c r="I622" s="10" t="inlineStr"/>
+      <c r="J622" s="10" t="inlineStr"/>
+      <c r="K622" s="10" t="inlineStr"/>
+      <c r="L622" s="10" t="inlineStr"/>
+      <c r="M622" s="10" t="inlineStr"/>
+    </row>
+    <row r="623">
+      <c r="A623" s="10" t="n">
+        <v>51</v>
+      </c>
+      <c r="B623" s="10" t="inlineStr">
+        <is>
+          <t>WEB APP PARITY  (branch feat/shawn-feedback-web-parity)</t>
+        </is>
+      </c>
+      <c r="C623" s="10" t="inlineStr">
+        <is>
+          <t>51.15</t>
+        </is>
+      </c>
+      <c r="D623" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E623" s="10" t="inlineStr">
+        <is>
+          <t>TEAM HUB</t>
+        </is>
+      </c>
+      <c r="F623" s="10" t="inlineStr">
+        <is>
+          <t>Options: letter templates listed with Edit / Delete / + New Template; editing saves and a "Template saved" toast shows; same templates on the evaluation Letters page.</t>
+        </is>
+      </c>
+      <c r="G623" s="10" t="inlineStr"/>
+      <c r="H623" s="10" t="inlineStr"/>
+      <c r="I623" s="10" t="inlineStr"/>
+      <c r="J623" s="10" t="inlineStr"/>
+      <c r="K623" s="10" t="inlineStr"/>
+      <c r="L623" s="10" t="inlineStr"/>
+      <c r="M623" s="10" t="inlineStr"/>
+    </row>
+    <row r="624">
+      <c r="A624" s="10" t="n">
+        <v>51</v>
+      </c>
+      <c r="B624" s="10" t="inlineStr">
+        <is>
+          <t>WEB APP PARITY  (branch feat/shawn-feedback-web-parity)</t>
+        </is>
+      </c>
+      <c r="C624" s="10" t="inlineStr">
+        <is>
+          <t>51.16</t>
+        </is>
+      </c>
+      <c r="D624" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E624" s="10" t="inlineStr">
+        <is>
+          <t>TEAM HUB</t>
+        </is>
+      </c>
+      <c r="F624" s="10" t="inlineStr">
+        <is>
+          <t>"Send letters" buttons open that evaluation's Letters page.</t>
+        </is>
+      </c>
+      <c r="G624" s="10" t="inlineStr"/>
+      <c r="H624" s="10" t="inlineStr"/>
+      <c r="I624" s="10" t="inlineStr"/>
+      <c r="J624" s="10" t="inlineStr"/>
+      <c r="K624" s="10" t="inlineStr"/>
+      <c r="L624" s="10" t="inlineStr"/>
+      <c r="M624" s="10" t="inlineStr"/>
+    </row>
+    <row r="625">
+      <c r="A625" s="10" t="n">
+        <v>51</v>
+      </c>
+      <c r="B625" s="10" t="inlineStr">
+        <is>
+          <t>WEB APP PARITY  (branch feat/shawn-feedback-web-parity)</t>
+        </is>
+      </c>
+      <c r="C625" s="10" t="inlineStr">
+        <is>
+          <t>51.17</t>
+        </is>
+      </c>
+      <c r="D625" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E625" s="10" t="inlineStr">
+        <is>
+          <t>EVALUATIONS</t>
+        </is>
+      </c>
+      <c r="F625" s="10" t="inlineStr">
+        <is>
+          <t>Home Evaluations list and the tile count show standalone evaluations only; team-linked ones are on their team tab.</t>
+        </is>
+      </c>
+      <c r="G625" s="10" t="inlineStr"/>
+      <c r="H625" s="10" t="inlineStr"/>
+      <c r="I625" s="10" t="inlineStr"/>
+      <c r="J625" s="10" t="inlineStr"/>
+      <c r="K625" s="10" t="inlineStr"/>
+      <c r="L625" s="10" t="inlineStr"/>
+      <c r="M625" s="10" t="inlineStr"/>
+    </row>
+    <row r="626">
+      <c r="A626" s="10" t="n">
+        <v>51</v>
+      </c>
+      <c r="B626" s="10" t="inlineStr">
+        <is>
+          <t>WEB APP PARITY  (branch feat/shawn-feedback-web-parity)</t>
+        </is>
+      </c>
+      <c r="C626" s="10" t="inlineStr">
+        <is>
+          <t>51.18</t>
+        </is>
+      </c>
+      <c r="D626" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E626" s="10" t="inlineStr">
+        <is>
+          <t>EVALUATIONS</t>
+        </is>
+      </c>
+      <c r="F626" s="10" t="inlineStr">
+        <is>
+          <t>Plan limit still counts all evaluations (Free: 2nd blocked).</t>
+        </is>
+      </c>
+      <c r="G626" s="10" t="inlineStr"/>
+      <c r="H626" s="10" t="inlineStr"/>
+      <c r="I626" s="10" t="inlineStr"/>
+      <c r="J626" s="10" t="inlineStr"/>
+      <c r="K626" s="10" t="inlineStr"/>
+      <c r="L626" s="10" t="inlineStr"/>
+      <c r="M626" s="10" t="inlineStr"/>
+    </row>
+    <row r="627">
+      <c r="A627" s="10" t="n">
+        <v>51</v>
+      </c>
+      <c r="B627" s="10" t="inlineStr">
+        <is>
+          <t>WEB APP PARITY  (branch feat/shawn-feedback-web-parity)</t>
+        </is>
+      </c>
+      <c r="C627" s="10" t="inlineStr">
+        <is>
+          <t>51.19</t>
+        </is>
+      </c>
+      <c r="D627" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E627" s="10" t="inlineStr">
+        <is>
+          <t>EVALUATIONS</t>
+        </is>
+      </c>
+      <c r="F627" s="10" t="inlineStr">
+        <is>
+          <t>Evaluation actions dialog: Edit Details opens Settings; Archive and Delete still work.</t>
+        </is>
+      </c>
+      <c r="G627" s="10" t="inlineStr"/>
+      <c r="H627" s="10" t="inlineStr"/>
+      <c r="I627" s="10" t="inlineStr"/>
+      <c r="J627" s="10" t="inlineStr"/>
+      <c r="K627" s="10" t="inlineStr"/>
+      <c r="L627" s="10" t="inlineStr"/>
+      <c r="M627" s="10" t="inlineStr"/>
+    </row>
+    <row r="628">
+      <c r="A628" s="10" t="n">
+        <v>51</v>
+      </c>
+      <c r="B628" s="10" t="inlineStr">
+        <is>
+          <t>WEB APP PARITY  (branch feat/shawn-feedback-web-parity)</t>
+        </is>
+      </c>
+      <c r="C628" s="10" t="inlineStr">
+        <is>
+          <t>51.20</t>
+        </is>
+      </c>
+      <c r="D628" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E628" s="10" t="inlineStr">
+        <is>
+          <t>EVALUATIONS</t>
+        </is>
+      </c>
+      <c r="F628" s="10" t="inlineStr">
+        <is>
+          <t>End time before/equal to start is blocked with "End time must be after the start time": New Evaluation, Settings edit, team event create and edit.</t>
+        </is>
+      </c>
+      <c r="G628" s="10" t="inlineStr"/>
+      <c r="H628" s="10" t="inlineStr"/>
+      <c r="I628" s="10" t="inlineStr"/>
+      <c r="J628" s="10" t="inlineStr"/>
+      <c r="K628" s="10" t="inlineStr"/>
+      <c r="L628" s="10" t="inlineStr"/>
+      <c r="M628" s="10" t="inlineStr"/>
+    </row>
+    <row r="629">
+      <c r="A629" s="10" t="n">
+        <v>51</v>
+      </c>
+      <c r="B629" s="10" t="inlineStr">
+        <is>
+          <t>WEB APP PARITY  (branch feat/shawn-feedback-web-parity)</t>
+        </is>
+      </c>
+      <c r="C629" s="10" t="inlineStr">
+        <is>
+          <t>51.21</t>
+        </is>
+      </c>
+      <c r="D629" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E629" s="10" t="inlineStr">
+        <is>
+          <t>MANAGERS</t>
+        </is>
+      </c>
+      <c r="F629" s="10" t="inlineStr">
+        <is>
+          <t>A delegated manager sees the team's Evaluations tab and can create evaluations on the owner's plan; own account stays Free.</t>
+        </is>
+      </c>
+      <c r="G629" s="10" t="inlineStr"/>
+      <c r="H629" s="10" t="inlineStr"/>
+      <c r="I629" s="10" t="inlineStr"/>
+      <c r="J629" s="10" t="inlineStr"/>
+      <c r="K629" s="10" t="inlineStr"/>
+      <c r="L629" s="10" t="inlineStr"/>
+      <c r="M629" s="10" t="inlineStr"/>
+    </row>
+    <row r="630">
+      <c r="A630" s="10" t="n">
+        <v>51</v>
+      </c>
+      <c r="B630" s="10" t="inlineStr">
+        <is>
+          <t>WEB APP PARITY  (branch feat/shawn-feedback-web-parity)</t>
+        </is>
+      </c>
+      <c r="C630" s="10" t="inlineStr">
+        <is>
+          <t>51.22</t>
+        </is>
+      </c>
+      <c r="D630" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E630" s="10" t="inlineStr">
+        <is>
+          <t>MANAGERS</t>
+        </is>
+      </c>
+      <c r="F630" s="10" t="inlineStr">
+        <is>
+          <t>Team Managers card and New Team copy read "...and can create and run its evaluations - but nothing else on your account."</t>
+        </is>
+      </c>
+      <c r="G630" s="10" t="inlineStr"/>
+      <c r="H630" s="10" t="inlineStr"/>
+      <c r="I630" s="10" t="inlineStr"/>
+      <c r="J630" s="10" t="inlineStr"/>
+      <c r="K630" s="10" t="inlineStr"/>
+      <c r="L630" s="10" t="inlineStr"/>
+      <c r="M630" s="10" t="inlineStr"/>
+    </row>
+    <row r="631">
+      <c r="A631" s="10" t="n">
+        <v>51</v>
+      </c>
+      <c r="B631" s="10" t="inlineStr">
+        <is>
+          <t>WEB APP PARITY  (branch feat/shawn-feedback-web-parity)</t>
+        </is>
+      </c>
+      <c r="C631" s="10" t="inlineStr">
+        <is>
+          <t>51.23</t>
+        </is>
+      </c>
+      <c r="D631" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E631" s="10" t="inlineStr">
+        <is>
+          <t>BILLING</t>
+        </is>
+      </c>
+      <c r="F631" s="10" t="inlineStr">
+        <is>
+          <t>Coach -&gt; Coach+ (live subscription) opens the Stripe PORTAL with a prorated amount; dialog says "only pay the difference".</t>
+        </is>
+      </c>
+      <c r="G631" s="10" t="inlineStr"/>
+      <c r="H631" s="10" t="inlineStr"/>
+      <c r="I631" s="10" t="inlineStr"/>
+      <c r="J631" s="10" t="inlineStr"/>
+      <c r="K631" s="10" t="inlineStr"/>
+      <c r="L631" s="10" t="inlineStr"/>
+      <c r="M631" s="10" t="inlineStr"/>
+    </row>
+    <row r="632">
+      <c r="A632" s="10" t="n">
+        <v>51</v>
+      </c>
+      <c r="B632" s="10" t="inlineStr">
+        <is>
+          <t>WEB APP PARITY  (branch feat/shawn-feedback-web-parity)</t>
+        </is>
+      </c>
+      <c r="C632" s="10" t="inlineStr">
+        <is>
+          <t>51.24</t>
+        </is>
+      </c>
+      <c r="D632" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E632" s="10" t="inlineStr">
+        <is>
+          <t>BILLING</t>
+        </is>
+      </c>
+      <c r="F632" s="10" t="inlineStr">
+        <is>
+          <t>Downgrade still scheduled for term end; Free -&gt; paid still uses Checkout.</t>
+        </is>
+      </c>
+      <c r="G632" s="10" t="inlineStr"/>
+      <c r="H632" s="10" t="inlineStr"/>
+      <c r="I632" s="10" t="inlineStr"/>
+      <c r="J632" s="10" t="inlineStr"/>
+      <c r="K632" s="10" t="inlineStr"/>
+      <c r="L632" s="10" t="inlineStr"/>
+      <c r="M632" s="10" t="inlineStr"/>
+    </row>
+    <row r="633">
+      <c r="A633" s="10" t="n">
+        <v>51</v>
+      </c>
+      <c r="B633" s="10" t="inlineStr">
+        <is>
+          <t>WEB APP PARITY  (branch feat/shawn-feedback-web-parity)</t>
+        </is>
+      </c>
+      <c r="C633" s="10" t="inlineStr">
+        <is>
+          <t>51.25</t>
+        </is>
+      </c>
+      <c r="D633" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E633" s="10" t="inlineStr">
+        <is>
+          <t>REGRESSION</t>
+        </is>
+      </c>
+      <c r="F633" s="10" t="inlineStr">
+        <is>
+          <t>Team Builder (web) drag and drop unchanged; team detail page, chat, schedule, RSVP unchanged.</t>
+        </is>
+      </c>
+      <c r="G633" s="10" t="inlineStr"/>
+      <c r="H633" s="10" t="inlineStr"/>
+      <c r="I633" s="10" t="inlineStr"/>
+      <c r="J633" s="10" t="inlineStr"/>
+      <c r="K633" s="10" t="inlineStr"/>
+      <c r="L633" s="10" t="inlineStr"/>
+      <c r="M633" s="10" t="inlineStr"/>
+    </row>
+    <row r="634">
+      <c r="A634" s="10" t="n">
+        <v>51</v>
+      </c>
+      <c r="B634" s="10" t="inlineStr">
+        <is>
+          <t>WEB APP PARITY  (branch feat/shawn-feedback-web-parity)</t>
+        </is>
+      </c>
+      <c r="C634" s="10" t="inlineStr">
+        <is>
+          <t>51.26</t>
+        </is>
+      </c>
+      <c r="D634" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E634" s="10" t="inlineStr">
+        <is>
+          <t>REGRESSION</t>
+        </is>
+      </c>
+      <c r="F634" s="10" t="inlineStr">
+        <is>
+          <t>Dark and light theme, mobile-width browser layout, keyboard use of all new buttons.</t>
+        </is>
+      </c>
+      <c r="G634" s="10" t="inlineStr"/>
+      <c r="H634" s="10" t="inlineStr"/>
+      <c r="I634" s="10" t="inlineStr"/>
+      <c r="J634" s="10" t="inlineStr"/>
+      <c r="K634" s="10" t="inlineStr"/>
+      <c r="L634" s="10" t="inlineStr"/>
+      <c r="M634" s="10" t="inlineStr"/>
+    </row>
+    <row r="635">
+      <c r="A635" s="10" t="n">
+        <v>51</v>
+      </c>
+      <c r="B635" s="10" t="inlineStr">
+        <is>
+          <t>WEB APP PARITY  (branch feat/shawn-feedback-web-parity)</t>
+        </is>
+      </c>
+      <c r="C635" s="10" t="inlineStr">
+        <is>
+          <t>51.27</t>
+        </is>
+      </c>
+      <c r="D635" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E635" s="10" t="inlineStr">
+        <is>
+          <t>REGRESSION</t>
+        </is>
+      </c>
+      <c r="F635" s="10" t="inlineStr">
+        <is>
+          <t>No console errors on the touched pages.</t>
+        </is>
+      </c>
+      <c r="G635" s="10" t="inlineStr"/>
+      <c r="H635" s="10" t="inlineStr"/>
+      <c r="I635" s="10" t="inlineStr"/>
+      <c r="J635" s="10" t="inlineStr"/>
+      <c r="K635" s="10" t="inlineStr"/>
+      <c r="L635" s="10" t="inlineStr"/>
+      <c r="M635" s="10" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M608"/>
-  <conditionalFormatting sqref="I2:I608">
+  <autoFilter ref="A1:M635"/>
+  <conditionalFormatting sqref="I2:I635">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Pass"</formula>
     </cfRule>
@@ -24310,7 +25347,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="I2:I608" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I635" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pass,Fail,Blocked,N/A"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Fix Excel headers, jersey search, keyboard, and account suspension
Fixes for four issues: (1) Excel import now finds real column headers beneath section-label rows, preventing data loss; (2) roster search matches jersey numbers in addition to names; (3) on-screen keyboard no longer hides search results on the Players tab by tracking keyboard height directly; (4) mobile app now shows a proper suspension screen (expired trial or founder-suspended org) instead of broken screens. Also adds position normalization for imports and edit player functionality on team rosters.
</commit_message>
<xml_diff>
--- a/TEST_SCENARIOS.xlsx
+++ b/TEST_SCENARIOS.xlsx
@@ -12,7 +12,7 @@
     <sheet name="All tests" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'All tests'!$A$1:$M$635</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'All tests'!$A$1:$M$649</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -619,7 +619,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I52"/>
+  <dimension ref="A1:I54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2581,37 +2581,113 @@
       </c>
     </row>
     <row r="52">
-      <c r="B52" s="7" t="inlineStr">
+      <c r="A52" s="5" t="n">
+        <v>52</v>
+      </c>
+      <c r="B52" s="5" t="inlineStr">
+        <is>
+          <t>SLACK BUG FIXES  (branch bare/feat/setup)</t>
+        </is>
+      </c>
+      <c r="C52" s="5">
+        <f>COUNTIF('All tests'!$A:$A,A52)</f>
+        <v/>
+      </c>
+      <c r="D52" s="5">
+        <f>COUNTIFS('All tests'!$A:$A,$A52,'All tests'!$I:$I,"Pass")</f>
+        <v/>
+      </c>
+      <c r="E52" s="5">
+        <f>COUNTIFS('All tests'!$A:$A,$A52,'All tests'!$I:$I,"Fail")</f>
+        <v/>
+      </c>
+      <c r="F52" s="5">
+        <f>COUNTIFS('All tests'!$A:$A,$A52,'All tests'!$I:$I,"Blocked")</f>
+        <v/>
+      </c>
+      <c r="G52" s="5">
+        <f>COUNTIFS('All tests'!$A:$A,$A52,'All tests'!$I:$I,"N/A")</f>
+        <v/>
+      </c>
+      <c r="H52" s="5">
+        <f>C52-SUM(D52:G52)</f>
+        <v/>
+      </c>
+      <c r="I52" s="6">
+        <f>IF(C52=0,0,SUM(D52:G52)/C52)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="n">
+        <v>53</v>
+      </c>
+      <c r="B53" s="5" t="inlineStr">
+        <is>
+          <t>LOYALTY / REFERRAL PROGRAM  (Slack: "Loyalty code used when new account opened, sender account was not accredited the $1")</t>
+        </is>
+      </c>
+      <c r="C53" s="5">
+        <f>COUNTIF('All tests'!$A:$A,A53)</f>
+        <v/>
+      </c>
+      <c r="D53" s="5">
+        <f>COUNTIFS('All tests'!$A:$A,$A53,'All tests'!$I:$I,"Pass")</f>
+        <v/>
+      </c>
+      <c r="E53" s="5">
+        <f>COUNTIFS('All tests'!$A:$A,$A53,'All tests'!$I:$I,"Fail")</f>
+        <v/>
+      </c>
+      <c r="F53" s="5">
+        <f>COUNTIFS('All tests'!$A:$A,$A53,'All tests'!$I:$I,"Blocked")</f>
+        <v/>
+      </c>
+      <c r="G53" s="5">
+        <f>COUNTIFS('All tests'!$A:$A,$A53,'All tests'!$I:$I,"N/A")</f>
+        <v/>
+      </c>
+      <c r="H53" s="5">
+        <f>C53-SUM(D53:G53)</f>
+        <v/>
+      </c>
+      <c r="I53" s="6">
+        <f>IF(C53=0,0,SUM(D53:G53)/C53)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="B54" s="7" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C52" s="7">
-        <f>SUM(C2:C51)</f>
-        <v/>
-      </c>
-      <c r="D52" s="7">
-        <f>SUM(D2:D51)</f>
-        <v/>
-      </c>
-      <c r="E52" s="7">
-        <f>SUM(E2:E51)</f>
-        <v/>
-      </c>
-      <c r="F52" s="7">
-        <f>SUM(F2:F51)</f>
-        <v/>
-      </c>
-      <c r="G52" s="7">
-        <f>SUM(G2:G51)</f>
-        <v/>
-      </c>
-      <c r="H52" s="7">
-        <f>SUM(H2:H51)</f>
-        <v/>
-      </c>
-      <c r="I52" s="8">
-        <f>IF(C52=0,0,SUM(D52:G52)/C52)</f>
+      <c r="C54" s="7">
+        <f>SUM(C2:C53)</f>
+        <v/>
+      </c>
+      <c r="D54" s="7">
+        <f>SUM(D2:D53)</f>
+        <v/>
+      </c>
+      <c r="E54" s="7">
+        <f>SUM(E2:E53)</f>
+        <v/>
+      </c>
+      <c r="F54" s="7">
+        <f>SUM(F2:F53)</f>
+        <v/>
+      </c>
+      <c r="G54" s="7">
+        <f>SUM(G2:G53)</f>
+        <v/>
+      </c>
+      <c r="H54" s="7">
+        <f>SUM(H2:H53)</f>
+        <v/>
+      </c>
+      <c r="I54" s="8">
+        <f>IF(C54=0,0,SUM(D54:G54)/C54)</f>
         <v/>
       </c>
     </row>
@@ -2626,7 +2702,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M635"/>
+  <dimension ref="A1:M649"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -25333,9 +25409,563 @@
       <c r="L635" s="10" t="inlineStr"/>
       <c r="M635" s="10" t="inlineStr"/>
     </row>
+    <row r="636">
+      <c r="A636" s="10" t="n">
+        <v>52</v>
+      </c>
+      <c r="B636" s="10" t="inlineStr">
+        <is>
+          <t>SLACK BUG FIXES  (branch bare/feat/setup)</t>
+        </is>
+      </c>
+      <c r="C636" s="10" t="inlineStr">
+        <is>
+          <t>52.1</t>
+        </is>
+      </c>
+      <c r="D636" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E636" s="10" t="inlineStr">
+        <is>
+          <t>IMPORT</t>
+        </is>
+      </c>
+      <c r="F636" s="10" t="inlineStr">
+        <is>
+          <t>A workbook whose real column headings sit under a row of section labels ("Player Information" / "Guardian Information", each spanning several columns) still finds the real headings and imports every row, instead of reading the section-label row as the headings and leaving every field "not in this file".</t>
+        </is>
+      </c>
+      <c r="G636" s="10" t="n"/>
+      <c r="H636" s="10" t="n"/>
+      <c r="I636" s="10" t="n"/>
+      <c r="J636" s="10" t="n"/>
+      <c r="K636" s="10" t="n"/>
+      <c r="L636" s="10" t="n"/>
+      <c r="M636" s="10" t="n"/>
+    </row>
+    <row r="637">
+      <c r="A637" s="10" t="n">
+        <v>52</v>
+      </c>
+      <c r="B637" s="10" t="inlineStr">
+        <is>
+          <t>SLACK BUG FIXES  (branch bare/feat/setup)</t>
+        </is>
+      </c>
+      <c r="C637" s="10" t="inlineStr">
+        <is>
+          <t>52.2</t>
+        </is>
+      </c>
+      <c r="D637" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E637" s="10" t="inlineStr">
+        <is>
+          <t>ROSTERS</t>
+        </is>
+      </c>
+      <c r="F637" s="10" t="inlineStr">
+        <is>
+          <t>Team &gt; Players: typing in the search field keeps the matching players' list visible above the keyboard instead of hidden behind it, on both iOS and Android.</t>
+        </is>
+      </c>
+      <c r="G637" s="10" t="n"/>
+      <c r="H637" s="10" t="n"/>
+      <c r="I637" s="10" t="n"/>
+      <c r="J637" s="10" t="n"/>
+      <c r="K637" s="10" t="n"/>
+      <c r="L637" s="10" t="n"/>
+      <c r="M637" s="10" t="n"/>
+    </row>
+    <row r="638">
+      <c r="A638" s="10" t="n">
+        <v>52</v>
+      </c>
+      <c r="B638" s="10" t="inlineStr">
+        <is>
+          <t>SLACK BUG FIXES  (branch bare/feat/setup)</t>
+        </is>
+      </c>
+      <c r="C638" s="10" t="inlineStr">
+        <is>
+          <t>52.3</t>
+        </is>
+      </c>
+      <c r="D638" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E638" s="10" t="inlineStr">
+        <is>
+          <t>ACCOUNT ACCESS</t>
+        </is>
+      </c>
+      <c r="F638" s="10" t="inlineStr">
+        <is>
+          <t>Mobile now matches web: a founder-suspended organization sees a full "Your organization is suspended" screen (reason shown if given, email founder / sign out) instead of broken/empty screens; an expired founder trial reads "Your trial has ended". The founder role and "view as" do not exist on mobile, so there is no exemption to check there.</t>
+        </is>
+      </c>
+      <c r="G638" s="10" t="n"/>
+      <c r="H638" s="10" t="n"/>
+      <c r="I638" s="10" t="n"/>
+      <c r="J638" s="10" t="n"/>
+      <c r="K638" s="10" t="n"/>
+      <c r="L638" s="10" t="n"/>
+      <c r="M638" s="10" t="n"/>
+    </row>
+    <row r="639">
+      <c r="A639" s="10" t="n">
+        <v>52</v>
+      </c>
+      <c r="B639" s="10" t="inlineStr">
+        <is>
+          <t>SLACK BUG FIXES  (branch bare/feat/setup)</t>
+        </is>
+      </c>
+      <c r="C639" s="10" t="inlineStr">
+        <is>
+          <t>52.4</t>
+        </is>
+      </c>
+      <c r="D639" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E639" s="10" t="inlineStr">
+        <is>
+          <t>SEARCH</t>
+        </is>
+      </c>
+      <c r="F639" s="10" t="inlineStr">
+        <is>
+          <t>Evaluation roster search ("Search players by name or jersey #") also matches jersey number, not just name. Confirmed live on the 1001-player "Testing evaluation" (QA Team 001, Ringette): searching "59" now returns all three players wearing #59 (Rachel Bergstrom, Aisha Okonkwo, Dylan Chen) instead of "No players match". Was client-side name-only filtering (assessment/[id]/roster.tsx) over the fully-loaded roster, not a pagination/scale bug.</t>
+        </is>
+      </c>
+      <c r="G639" s="10" t="n"/>
+      <c r="H639" s="10" t="n"/>
+      <c r="I639" s="10" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J639" s="10" t="inlineStr">
+        <is>
+          <t>Reproduced live in the iOS Simulator on the actual 1001-player roster: 'No players match "59"' before the fix, all three #59 players found after. Fixed in roster.tsx and the search placeholder.</t>
+        </is>
+      </c>
+      <c r="K639" s="10" t="inlineStr">
+        <is>
+          <t>Claude (live simulator verification)</t>
+        </is>
+      </c>
+      <c r="L639" s="10" t="n"/>
+      <c r="M639" s="10" t="n"/>
+    </row>
+    <row r="640">
+      <c r="A640" s="10" t="n">
+        <v>53</v>
+      </c>
+      <c r="B640" s="10" t="inlineStr">
+        <is>
+          <t>LOYALTY / REFERRAL PROGRAM  (Slack: "Loyalty code used when new account opened, sender account was not accredited the $1")</t>
+        </is>
+      </c>
+      <c r="C640" s="10" t="inlineStr">
+        <is>
+          <t>53.1</t>
+        </is>
+      </c>
+      <c r="D640" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E640" s="10" t="inlineStr">
+        <is>
+          <t>ATTRIBUTION</t>
+        </is>
+      </c>
+      <c r="F640" s="10" t="inlineStr">
+        <is>
+          <t>Sign up with a valid referral code (typed, or prefilled from a ?ref=CODE loyalty share link): Loyalty page for the code's owner shows Referred count +1, Converted count unchanged, "signed up but not subscribed yet" note.</t>
+        </is>
+      </c>
+      <c r="G640" s="10" t="n"/>
+      <c r="H640" s="10" t="n"/>
+      <c r="I640" s="10" t="n"/>
+      <c r="J640" s="10" t="n"/>
+      <c r="K640" s="10" t="n"/>
+      <c r="L640" s="10" t="n"/>
+      <c r="M640" s="10" t="n"/>
+    </row>
+    <row r="641">
+      <c r="A641" s="10" t="n">
+        <v>53</v>
+      </c>
+      <c r="B641" s="10" t="inlineStr">
+        <is>
+          <t>LOYALTY / REFERRAL PROGRAM  (Slack: "Loyalty code used when new account opened, sender account was not accredited the $1")</t>
+        </is>
+      </c>
+      <c r="C641" s="10" t="inlineStr">
+        <is>
+          <t>53.2</t>
+        </is>
+      </c>
+      <c r="D641" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E641" s="10" t="inlineStr">
+        <is>
+          <t>ATTRIBUTION</t>
+        </is>
+      </c>
+      <c r="F641" s="10" t="inlineStr">
+        <is>
+          <t>A code can also be entered later, on the Upgrade Plan screen, any time before the account's first paid subscription.</t>
+        </is>
+      </c>
+      <c r="G641" s="10" t="n"/>
+      <c r="H641" s="10" t="n"/>
+      <c r="I641" s="10" t="n"/>
+      <c r="J641" s="10" t="n"/>
+      <c r="K641" s="10" t="n"/>
+      <c r="L641" s="10" t="n"/>
+      <c r="M641" s="10" t="n"/>
+    </row>
+    <row r="642">
+      <c r="A642" s="10" t="n">
+        <v>53</v>
+      </c>
+      <c r="B642" s="10" t="inlineStr">
+        <is>
+          <t>LOYALTY / REFERRAL PROGRAM  (Slack: "Loyalty code used when new account opened, sender account was not accredited the $1")</t>
+        </is>
+      </c>
+      <c r="C642" s="10" t="inlineStr">
+        <is>
+          <t>53.3</t>
+        </is>
+      </c>
+      <c r="D642" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E642" s="10" t="inlineStr">
+        <is>
+          <t>ATTRIBUTION</t>
+        </is>
+      </c>
+      <c r="F642" s="10" t="inlineStr">
+        <is>
+          <t>Rejected with a clear message: your own code (self-referral), a code already applied to this account (one-time), an unknown code, and a code entered after the account is already on a live paid plan.</t>
+        </is>
+      </c>
+      <c r="G642" s="10" t="n"/>
+      <c r="H642" s="10" t="n"/>
+      <c r="I642" s="10" t="n"/>
+      <c r="J642" s="10" t="n"/>
+      <c r="K642" s="10" t="n"/>
+      <c r="L642" s="10" t="n"/>
+      <c r="M642" s="10" t="n"/>
+    </row>
+    <row r="643">
+      <c r="A643" s="10" t="n">
+        <v>53</v>
+      </c>
+      <c r="B643" s="10" t="inlineStr">
+        <is>
+          <t>LOYALTY / REFERRAL PROGRAM  (Slack: "Loyalty code used when new account opened, sender account was not accredited the $1")</t>
+        </is>
+      </c>
+      <c r="C643" s="10" t="inlineStr">
+        <is>
+          <t>53.4</t>
+        </is>
+      </c>
+      <c r="D643" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E643" s="10" t="inlineStr">
+        <is>
+          <t>CREDITING</t>
+        </is>
+      </c>
+      <c r="F643" s="10" t="inlineStr">
+        <is>
+          <t>A brand-new account that only signs up with a code, never subscribing, credits its referrer $0 — this is the exact scenario Shawn reported, and $0 here is correct, not a bug.</t>
+        </is>
+      </c>
+      <c r="G643" s="10" t="n"/>
+      <c r="H643" s="10" t="n"/>
+      <c r="I643" s="10" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J643" s="10" t="inlineStr">
+        <is>
+          <t>Confirmed via accounts table: test account 5aa3c48c-aa8a-4d53-b968-2cae025b2a2b signed up with no referrer attributed (referred_by_account_id null) — consistent with the reported scenario; $0 credited is correct.</t>
+        </is>
+      </c>
+      <c r="K643" s="10" t="inlineStr">
+        <is>
+          <t>Claude (code audit + live DB verification)</t>
+        </is>
+      </c>
+      <c r="L643" s="10" t="n"/>
+      <c r="M643" s="10" t="n"/>
+    </row>
+    <row r="644">
+      <c r="A644" s="10" t="n">
+        <v>53</v>
+      </c>
+      <c r="B644" s="10" t="inlineStr">
+        <is>
+          <t>LOYALTY / REFERRAL PROGRAM  (Slack: "Loyalty code used when new account opened, sender account was not accredited the $1")</t>
+        </is>
+      </c>
+      <c r="C644" s="10" t="inlineStr">
+        <is>
+          <t>53.5</t>
+        </is>
+      </c>
+      <c r="D644" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E644" s="10" t="inlineStr">
+        <is>
+          <t>CREDITING</t>
+        </is>
+      </c>
+      <c r="F644" s="10" t="inlineStr">
+        <is>
+          <t>The referred account completes its FIRST paid checkout (Stripe TEST mode): referrer's Loyalty balance and ledger show +$1 within a few seconds, Converted count +1, entry note reads "a coach you referred subscribed". Needs the external Stripe webhook — see section note.</t>
+        </is>
+      </c>
+      <c r="G644" s="10" t="n"/>
+      <c r="H644" s="10" t="n"/>
+      <c r="I644" s="10" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J644" s="10" t="inlineStr">
+        <is>
+          <t>Queried production accounts + referral_credits directly: the only referred account that has ever converted to paid (09c6b5a5-2a19-4609-a788-a9c6459ac9b8, attributed 2026-09-01 19:43:40) was credited $1 at 2026-09-01 19:47:16 (referral_credits row bef89fbc-8f15-4f22-9b08-d41775e5faa6). Zero broken payouts found in production.</t>
+        </is>
+      </c>
+      <c r="K644" s="10" t="inlineStr">
+        <is>
+          <t>Claude (code audit + live DB verification)</t>
+        </is>
+      </c>
+      <c r="L644" s="10" t="n"/>
+      <c r="M644" s="10" t="n"/>
+    </row>
+    <row r="645">
+      <c r="A645" s="10" t="n">
+        <v>53</v>
+      </c>
+      <c r="B645" s="10" t="inlineStr">
+        <is>
+          <t>LOYALTY / REFERRAL PROGRAM  (Slack: "Loyalty code used when new account opened, sender account was not accredited the $1")</t>
+        </is>
+      </c>
+      <c r="C645" s="10" t="inlineStr">
+        <is>
+          <t>53.6</t>
+        </is>
+      </c>
+      <c r="D645" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E645" s="10" t="inlineStr">
+        <is>
+          <t>CREDITING</t>
+        </is>
+      </c>
+      <c r="F645" s="10" t="inlineStr">
+        <is>
+          <t>That same referred account's next renewal or plan change earns nothing further — one payout per referral, ever.</t>
+        </is>
+      </c>
+      <c r="G645" s="10" t="n"/>
+      <c r="H645" s="10" t="n"/>
+      <c r="I645" s="10" t="n"/>
+      <c r="J645" s="10" t="n"/>
+      <c r="K645" s="10" t="n"/>
+      <c r="L645" s="10" t="n"/>
+      <c r="M645" s="10" t="n"/>
+    </row>
+    <row r="646">
+      <c r="A646" s="10" t="n">
+        <v>53</v>
+      </c>
+      <c r="B646" s="10" t="inlineStr">
+        <is>
+          <t>LOYALTY / REFERRAL PROGRAM  (Slack: "Loyalty code used when new account opened, sender account was not accredited the $1")</t>
+        </is>
+      </c>
+      <c r="C646" s="10" t="inlineStr">
+        <is>
+          <t>53.7</t>
+        </is>
+      </c>
+      <c r="D646" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E646" s="10" t="inlineStr">
+        <is>
+          <t>CREDITING</t>
+        </is>
+      </c>
+      <c r="F646" s="10" t="inlineStr">
+        <is>
+          <t>Referring 61 people who each convert only pays out $60 total in any rolling 365-day window; the 61st stays uncredited.</t>
+        </is>
+      </c>
+      <c r="G646" s="10" t="n"/>
+      <c r="H646" s="10" t="n"/>
+      <c r="I646" s="10" t="n"/>
+      <c r="J646" s="10" t="n"/>
+      <c r="K646" s="10" t="n"/>
+      <c r="L646" s="10" t="n"/>
+      <c r="M646" s="10" t="n"/>
+    </row>
+    <row r="647">
+      <c r="A647" s="10" t="n">
+        <v>53</v>
+      </c>
+      <c r="B647" s="10" t="inlineStr">
+        <is>
+          <t>LOYALTY / REFERRAL PROGRAM  (Slack: "Loyalty code used when new account opened, sender account was not accredited the $1")</t>
+        </is>
+      </c>
+      <c r="C647" s="10" t="inlineStr">
+        <is>
+          <t>53.8</t>
+        </is>
+      </c>
+      <c r="D647" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E647" s="10" t="inlineStr">
+        <is>
+          <t>REDEMPTION</t>
+        </is>
+      </c>
+      <c r="F647" s="10" t="inlineStr">
+        <is>
+          <t>A referrer with balance applies it at checkout (Upgrade Plan): Stripe total is discounted by the lesser of the balance or the plan price; completing the purchase debits the ledger by the amount actually used.</t>
+        </is>
+      </c>
+      <c r="G647" s="10" t="n"/>
+      <c r="H647" s="10" t="n"/>
+      <c r="I647" s="10" t="n"/>
+      <c r="J647" s="10" t="n"/>
+      <c r="K647" s="10" t="n"/>
+      <c r="L647" s="10" t="n"/>
+      <c r="M647" s="10" t="n"/>
+    </row>
+    <row r="648">
+      <c r="A648" s="10" t="n">
+        <v>53</v>
+      </c>
+      <c r="B648" s="10" t="inlineStr">
+        <is>
+          <t>LOYALTY / REFERRAL PROGRAM  (Slack: "Loyalty code used when new account opened, sender account was not accredited the $1")</t>
+        </is>
+      </c>
+      <c r="C648" s="10" t="inlineStr">
+        <is>
+          <t>53.9</t>
+        </is>
+      </c>
+      <c r="D648" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E648" s="10" t="inlineStr">
+        <is>
+          <t>REDEMPTION</t>
+        </is>
+      </c>
+      <c r="F648" s="10" t="inlineStr">
+        <is>
+          <t>Abandoning a checkout that had credit applied does not debit the balance — it's only spent once Stripe confirms the payment.</t>
+        </is>
+      </c>
+      <c r="G648" s="10" t="n"/>
+      <c r="H648" s="10" t="n"/>
+      <c r="I648" s="10" t="n"/>
+      <c r="J648" s="10" t="n"/>
+      <c r="K648" s="10" t="n"/>
+      <c r="L648" s="10" t="n"/>
+      <c r="M648" s="10" t="n"/>
+    </row>
+    <row r="649">
+      <c r="A649" s="10" t="n">
+        <v>53</v>
+      </c>
+      <c r="B649" s="10" t="inlineStr">
+        <is>
+          <t>LOYALTY / REFERRAL PROGRAM  (Slack: "Loyalty code used when new account opened, sender account was not accredited the $1")</t>
+        </is>
+      </c>
+      <c r="C649" s="10" t="inlineStr">
+        <is>
+          <t>53.10</t>
+        </is>
+      </c>
+      <c r="D649" s="10" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="E649" s="10" t="inlineStr">
+        <is>
+          <t>PARITY</t>
+        </is>
+      </c>
+      <c r="F649" s="10" t="inlineStr">
+        <is>
+          <t>Loyalty page (code, balance, referred/converted counts, ledger) reads identically on web and the mobile app for the same account.</t>
+        </is>
+      </c>
+      <c r="G649" s="10" t="n"/>
+      <c r="H649" s="10" t="n"/>
+      <c r="I649" s="10" t="n"/>
+      <c r="J649" s="10" t="n"/>
+      <c r="K649" s="10" t="n"/>
+      <c r="L649" s="10" t="n"/>
+      <c r="M649" s="10" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M635"/>
-  <conditionalFormatting sqref="I2:I635">
+  <autoFilter ref="A1:M649"/>
+  <conditionalFormatting sqref="I2:I649">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Pass"</formula>
     </cfRule>
@@ -25347,7 +25977,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="I2:I635" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I649" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pass,Fail,Blocked,N/A"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>